<commit_message>
feat: make expert id optional — auto-generate seed_id on upload
Remove id from required columns in expert upload. If id is not
provided in the file, auto-generate seed_id (auto-{uuid8}).
Update experts XLSX template to remove id column.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/templates/experts_template.xlsx
+++ b/frontend/public/templates/experts_template.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Эксперты" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,8 +26,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -68,16 +72,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="00E5E7EB"/>
       </left>
       <right style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="00E5E7EB"/>
       </right>
       <top style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="00E5E7EB"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D1D5DB"/>
+        <color rgb="00E5E7EB"/>
       </bottom>
     </border>
   </borders>
@@ -89,12 +93,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -460,38 +460,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>id *</t>
+          <t>name *</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>name *</t>
+          <t>telegram</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>telegram</t>
+          <t>position</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>position</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>expertise_tags</t>
         </is>
@@ -500,25 +494,20 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>exp-001</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
           <t>Иванов Иван</t>
         </is>
       </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>@ivanov</t>
+        </is>
+      </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>@ivanov</t>
+          <t>Senior ML Engineer</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Senior ML Engineer</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>NLP, LLM, Chatbot</t>
         </is>
@@ -527,148 +516,22 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>exp-002</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
           <t>Петрова Мария</t>
         </is>
       </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>@petrova</t>
+        </is>
+      </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>@petrova</t>
+          <t>Data Scientist</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
           <t>CV, Detection, Segmentation</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Поле</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Обязательное</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Описание</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Уникальный идентификатор эксперта</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>ФИО эксперта</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>telegram</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Нет</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Telegram username (@username)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>position</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Нет</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Должность</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>expertise_tags</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Нет</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Теги экспертизы через запятую</t>
         </is>
       </c>
     </row>

</xml_diff>